<commit_message>
Improve complex BOM parsing and template output
</commit_message>
<xml_diff>
--- a/public/templates/bom-input-output-template.xlsx
+++ b/public/templates/bom-input-output-template.xlsx
@@ -1,34 +1,51 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
-  <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12375" activeTab="1"/>
-  </bookViews>
-  <sheets>
-    <sheet name="输入" sheetId="1" r:id="rId1"/>
-    <sheet name="输出" sheetId="2" r:id="rId2"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>WPS 表格</Application>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>工作表</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>2</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="2" baseType="lpstr">
+      <vt:lpstr>输入</vt:lpstr>
+      <vt:lpstr>输出</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="64">
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>admin</dc:creator>
+  <cp:lastModifiedBy>NiuMch</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-07-14T01:52:00Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-07-15T08:04:52Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="2" name="ICV">
+    <vt:lpwstr>2FF7BAB307B44F93859A54BB734C2917_11</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="KSOProductBuildVer">
+    <vt:lpwstr>2052-12.1.0.26391</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4" name="CalculationRule">
+    <vt:i4>1</vt:i4>
+  </property>
+</Properties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="66">
   <si>
     <t>供应商-产品名-型号-颜色（xxx-风扇灯-36寸智能-白色）</t>
   </si>
@@ -210,7 +227,13 @@
     <t>‘供应商1’</t>
   </si>
   <si>
+    <t>‘供应商1’规格描述</t>
+  </si>
+  <si>
     <t>‘供应商2’</t>
+  </si>
+  <si>
+    <t>‘供应商2’规格描述</t>
   </si>
   <si>
     <t>差价</t>
@@ -224,7 +247,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
@@ -994,7 +1017,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1028,9 +1051,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1082,14 +1102,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" quotePrefix="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" quotePrefix="1">
       <alignment vertical="center"/>
@@ -1373,7 +1387,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="WPS">
   <a:themeElements>
     <a:clrScheme name="WPS">
@@ -1620,7 +1634,34 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="28800" windowHeight="12375" activeTab="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="输入" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F67"/>
@@ -1633,37 +1674,37 @@
   </cols>
   <sheetData>
     <row r="1" ht="75" customHeight="1" spans="1:6">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" ht="23" customHeight="1" spans="1:6">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="23" t="s">
+      <c r="C2" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="23" t="s">
+      <c r="D2" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="23" t="s">
+      <c r="E2" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="23" t="s">
+      <c r="F2" s="22" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" ht="23" customHeight="1" spans="1:6">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="24" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="6" t="s">
@@ -1675,7 +1716,7 @@
       <c r="F3" s="7"/>
     </row>
     <row r="4" ht="23" customHeight="1" spans="1:6">
-      <c r="A4" s="25"/>
+      <c r="A4" s="24"/>
       <c r="B4" s="6" t="s">
         <v>9</v>
       </c>
@@ -1685,7 +1726,7 @@
       <c r="F4" s="7"/>
     </row>
     <row r="5" ht="23" customHeight="1" spans="1:6">
-      <c r="A5" s="25"/>
+      <c r="A5" s="24"/>
       <c r="B5" s="6" t="s">
         <v>10</v>
       </c>
@@ -1695,7 +1736,7 @@
       <c r="F5" s="7"/>
     </row>
     <row r="6" ht="23" customHeight="1" spans="1:6">
-      <c r="A6" s="25"/>
+      <c r="A6" s="24"/>
       <c r="B6" s="6" t="s">
         <v>11</v>
       </c>
@@ -1705,7 +1746,7 @@
       <c r="F6" s="7"/>
     </row>
     <row r="7" ht="23" customHeight="1" spans="1:6">
-      <c r="A7" s="25"/>
+      <c r="A7" s="24"/>
       <c r="B7" s="6" t="s">
         <v>12</v>
       </c>
@@ -1715,7 +1756,7 @@
       <c r="F7" s="7"/>
     </row>
     <row r="8" ht="23" customHeight="1" spans="1:6">
-      <c r="A8" s="25"/>
+      <c r="A8" s="24"/>
       <c r="B8" s="6" t="s">
         <v>13</v>
       </c>
@@ -1725,7 +1766,7 @@
       <c r="F8" s="7"/>
     </row>
     <row r="9" ht="23" customHeight="1" spans="1:6">
-      <c r="A9" s="25"/>
+      <c r="A9" s="24"/>
       <c r="B9" s="6" t="s">
         <v>14</v>
       </c>
@@ -1735,7 +1776,7 @@
       <c r="F9" s="7"/>
     </row>
     <row r="10" ht="23" customHeight="1" spans="1:6">
-      <c r="A10" s="25"/>
+      <c r="A10" s="24"/>
       <c r="B10" s="6" t="s">
         <v>15</v>
       </c>
@@ -1745,7 +1786,7 @@
       <c r="F10" s="7"/>
     </row>
     <row r="11" ht="23" customHeight="1" spans="1:6">
-      <c r="A11" s="25"/>
+      <c r="A11" s="24"/>
       <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
@@ -1755,7 +1796,7 @@
       <c r="F11" s="7"/>
     </row>
     <row r="12" ht="23" customHeight="1" spans="1:6">
-      <c r="A12" s="25"/>
+      <c r="A12" s="24"/>
       <c r="B12" s="6" t="s">
         <v>17</v>
       </c>
@@ -1765,7 +1806,7 @@
       <c r="F12" s="7"/>
     </row>
     <row r="13" ht="23" customHeight="1" spans="1:6">
-      <c r="A13" s="25"/>
+      <c r="A13" s="24"/>
       <c r="B13" s="6" t="s">
         <v>18</v>
       </c>
@@ -1775,7 +1816,7 @@
       <c r="F13" s="7"/>
     </row>
     <row r="14" ht="23" customHeight="1" spans="1:6">
-      <c r="A14" s="25"/>
+      <c r="A14" s="24"/>
       <c r="B14" s="6" t="s">
         <v>19</v>
       </c>
@@ -1785,7 +1826,7 @@
       <c r="F14" s="7"/>
     </row>
     <row r="15" ht="23" customHeight="1" spans="1:6">
-      <c r="A15" s="25"/>
+      <c r="A15" s="24"/>
       <c r="B15" s="6"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -1793,7 +1834,7 @@
       <c r="F15" s="7"/>
     </row>
     <row r="16" ht="23" customHeight="1" spans="1:6">
-      <c r="A16" s="25"/>
+      <c r="A16" s="24"/>
       <c r="B16" s="6"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
@@ -1801,14 +1842,14 @@
       <c r="F16" s="7"/>
     </row>
     <row r="17" ht="23" customHeight="1" spans="1:6">
-      <c r="A17" s="25"/>
-      <c r="C17" s="11"/>
+      <c r="A17" s="24"/>
+      <c r="C17" s="7"/>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
     </row>
     <row r="18" ht="23" customHeight="1" spans="1:6">
-      <c r="A18" s="25"/>
+      <c r="A18" s="24"/>
       <c r="B18" s="6"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
@@ -1816,7 +1857,7 @@
       <c r="F18" s="7"/>
     </row>
     <row r="19" ht="23" customHeight="1" spans="1:6">
-      <c r="A19" s="25"/>
+      <c r="A19" s="24"/>
       <c r="B19" s="6"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
@@ -1824,7 +1865,7 @@
       <c r="F19" s="7"/>
     </row>
     <row r="20" ht="23" customHeight="1" spans="1:6">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="24" t="s">
         <v>20</v>
       </c>
       <c r="B20" s="6" t="s">
@@ -1836,7 +1877,7 @@
       <c r="F20" s="7"/>
     </row>
     <row r="21" ht="23" customHeight="1" spans="1:6">
-      <c r="A21" s="25"/>
+      <c r="A21" s="24"/>
       <c r="B21" s="6" t="s">
         <v>22</v>
       </c>
@@ -1846,7 +1887,7 @@
       <c r="F21" s="7"/>
     </row>
     <row r="22" ht="23" customHeight="1" spans="1:6">
-      <c r="A22" s="25"/>
+      <c r="A22" s="24"/>
       <c r="B22" s="6" t="s">
         <v>23</v>
       </c>
@@ -1856,7 +1897,7 @@
       <c r="F22" s="7"/>
     </row>
     <row r="23" ht="23" customHeight="1" spans="1:6">
-      <c r="A23" s="25"/>
+      <c r="A23" s="24"/>
       <c r="B23" s="6" t="s">
         <v>24</v>
       </c>
@@ -1866,7 +1907,7 @@
       <c r="F23" s="7"/>
     </row>
     <row r="24" ht="23" customHeight="1" spans="1:6">
-      <c r="A24" s="25"/>
+      <c r="A24" s="24"/>
       <c r="B24" s="6" t="s">
         <v>25</v>
       </c>
@@ -1876,7 +1917,7 @@
       <c r="F24" s="7"/>
     </row>
     <row r="25" ht="23" customHeight="1" spans="1:6">
-      <c r="A25" s="25"/>
+      <c r="A25" s="24"/>
       <c r="B25" s="6" t="s">
         <v>26</v>
       </c>
@@ -1886,7 +1927,7 @@
       <c r="F25" s="7"/>
     </row>
     <row r="26" ht="23" customHeight="1" spans="1:6">
-      <c r="A26" s="25"/>
+      <c r="A26" s="24"/>
       <c r="B26" s="6" t="s">
         <v>23</v>
       </c>
@@ -1896,14 +1937,14 @@
       <c r="F26" s="7"/>
     </row>
     <row r="27" ht="23" customHeight="1" spans="1:6">
-      <c r="A27" s="25"/>
-      <c r="C27" s="11"/>
+      <c r="A27" s="24"/>
+      <c r="C27" s="7"/>
       <c r="D27" s="7"/>
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
     </row>
     <row r="28" ht="23" customHeight="1" spans="1:6">
-      <c r="A28" s="25"/>
+      <c r="A28" s="24"/>
       <c r="B28" s="6"/>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
@@ -1911,7 +1952,7 @@
       <c r="F28" s="7"/>
     </row>
     <row r="29" ht="23" customHeight="1" spans="1:6">
-      <c r="A29" s="26" t="s">
+      <c r="A29" s="25" t="s">
         <v>27</v>
       </c>
       <c r="B29" s="6" t="s">
@@ -1923,7 +1964,7 @@
       <c r="F29" s="7"/>
     </row>
     <row r="30" ht="23" customHeight="1" spans="1:6">
-      <c r="A30" s="27"/>
+      <c r="A30" s="26"/>
       <c r="B30" s="6" t="s">
         <v>29</v>
       </c>
@@ -1933,7 +1974,7 @@
       <c r="F30" s="7"/>
     </row>
     <row r="31" ht="23" customHeight="1" spans="1:6">
-      <c r="A31" s="27"/>
+      <c r="A31" s="26"/>
       <c r="B31" s="6" t="s">
         <v>30</v>
       </c>
@@ -1943,7 +1984,7 @@
       <c r="F31" s="7"/>
     </row>
     <row r="32" ht="23" customHeight="1" spans="1:6">
-      <c r="A32" s="27"/>
+      <c r="A32" s="26"/>
       <c r="B32" s="6"/>
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
@@ -1951,7 +1992,7 @@
       <c r="F32" s="7"/>
     </row>
     <row r="33" ht="23" customHeight="1" spans="1:6">
-      <c r="A33" s="27"/>
+      <c r="A33" s="26"/>
       <c r="B33" s="6"/>
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
@@ -1959,7 +2000,7 @@
       <c r="F33" s="7"/>
     </row>
     <row r="34" ht="23" customHeight="1" spans="1:6">
-      <c r="A34" s="28"/>
+      <c r="A34" s="27"/>
       <c r="B34" s="6"/>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
@@ -1967,7 +2008,7 @@
       <c r="F34" s="7"/>
     </row>
     <row r="35" ht="23" customHeight="1" spans="1:6">
-      <c r="A35" s="26" t="s">
+      <c r="A35" s="25" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="6" t="s">
@@ -1979,7 +2020,7 @@
       <c r="F35" s="7"/>
     </row>
     <row r="36" ht="23" customHeight="1" spans="1:6">
-      <c r="A36" s="27"/>
+      <c r="A36" s="26"/>
       <c r="B36" s="6" t="s">
         <v>33</v>
       </c>
@@ -1989,7 +2030,7 @@
       <c r="F36" s="7"/>
     </row>
     <row r="37" ht="23" customHeight="1" spans="1:6">
-      <c r="A37" s="27"/>
+      <c r="A37" s="26"/>
       <c r="B37" s="6" t="s">
         <v>34</v>
       </c>
@@ -1999,7 +2040,7 @@
       <c r="F37" s="7"/>
     </row>
     <row r="38" ht="23" customHeight="1" spans="1:6">
-      <c r="A38" s="27"/>
+      <c r="A38" s="26"/>
       <c r="B38" s="6" t="s">
         <v>34</v>
       </c>
@@ -2009,7 +2050,7 @@
       <c r="F38" s="7"/>
     </row>
     <row r="39" ht="23" customHeight="1" spans="1:6">
-      <c r="A39" s="27"/>
+      <c r="A39" s="26"/>
       <c r="B39" s="6" t="s">
         <v>35</v>
       </c>
@@ -2019,7 +2060,7 @@
       <c r="F39" s="7"/>
     </row>
     <row r="40" ht="23" customHeight="1" spans="1:6">
-      <c r="A40" s="27"/>
+      <c r="A40" s="26"/>
       <c r="B40" s="6" t="s">
         <v>36</v>
       </c>
@@ -2029,7 +2070,7 @@
       <c r="F40" s="7"/>
     </row>
     <row r="41" ht="23" customHeight="1" spans="1:6">
-      <c r="A41" s="27"/>
+      <c r="A41" s="26"/>
       <c r="B41" s="6"/>
       <c r="C41" s="7"/>
       <c r="D41" s="7"/>
@@ -2037,7 +2078,7 @@
       <c r="F41" s="7"/>
     </row>
     <row r="42" ht="23" customHeight="1" spans="1:6">
-      <c r="A42" s="27"/>
+      <c r="A42" s="26"/>
       <c r="B42" s="6"/>
       <c r="C42" s="7"/>
       <c r="D42" s="7"/>
@@ -2045,7 +2086,7 @@
       <c r="F42" s="7"/>
     </row>
     <row r="43" ht="23" customHeight="1" spans="1:6">
-      <c r="A43" s="27"/>
+      <c r="A43" s="26"/>
       <c r="B43" s="6"/>
       <c r="C43" s="7"/>
       <c r="D43" s="7"/>
@@ -2053,7 +2094,7 @@
       <c r="F43" s="7"/>
     </row>
     <row r="44" ht="23" customHeight="1" spans="1:6">
-      <c r="A44" s="27"/>
+      <c r="A44" s="26"/>
       <c r="B44" s="6"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -2061,7 +2102,7 @@
       <c r="F44" s="7"/>
     </row>
     <row r="45" ht="23" customHeight="1" spans="1:6">
-      <c r="A45" s="27"/>
+      <c r="A45" s="26"/>
       <c r="B45" s="6"/>
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
@@ -2069,7 +2110,7 @@
       <c r="F45" s="7"/>
     </row>
     <row r="46" ht="23" customHeight="1" spans="1:6">
-      <c r="A46" s="27"/>
+      <c r="A46" s="26"/>
       <c r="B46" s="6"/>
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
@@ -2077,7 +2118,7 @@
       <c r="F46" s="7"/>
     </row>
     <row r="47" ht="23" customHeight="1" spans="1:6">
-      <c r="A47" s="28"/>
+      <c r="A47" s="27"/>
       <c r="B47" s="6"/>
       <c r="C47" s="7"/>
       <c r="D47" s="7"/>
@@ -2085,7 +2126,7 @@
       <c r="F47" s="7"/>
     </row>
     <row r="48" ht="23" customHeight="1" spans="1:6">
-      <c r="A48" s="26" t="s">
+      <c r="A48" s="25" t="s">
         <v>37</v>
       </c>
       <c r="B48" s="6" t="s">
@@ -2097,7 +2138,7 @@
       <c r="F48" s="7"/>
     </row>
     <row r="49" ht="23" customHeight="1" spans="1:6">
-      <c r="A49" s="27"/>
+      <c r="A49" s="26"/>
       <c r="B49" s="6" t="s">
         <v>39</v>
       </c>
@@ -2107,7 +2148,7 @@
       <c r="F49" s="7"/>
     </row>
     <row r="50" ht="23" customHeight="1" spans="1:6">
-      <c r="A50" s="27"/>
+      <c r="A50" s="26"/>
       <c r="B50" s="6" t="s">
         <v>40</v>
       </c>
@@ -2117,7 +2158,7 @@
       <c r="F50" s="7"/>
     </row>
     <row r="51" ht="23" customHeight="1" spans="1:6">
-      <c r="A51" s="27"/>
+      <c r="A51" s="26"/>
       <c r="B51" s="6" t="s">
         <v>41</v>
       </c>
@@ -2127,7 +2168,7 @@
       <c r="F51" s="7"/>
     </row>
     <row r="52" ht="23" customHeight="1" spans="1:6">
-      <c r="A52" s="28"/>
+      <c r="A52" s="27"/>
       <c r="B52" s="6"/>
       <c r="C52" s="7"/>
       <c r="D52" s="7"/>
@@ -2135,10 +2176,10 @@
       <c r="F52" s="7"/>
     </row>
     <row r="53" ht="23" customHeight="1" spans="1:6">
-      <c r="A53" s="26" t="s">
+      <c r="A53" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="B53" s="31" t="s">
+      <c r="B53" s="29" t="s">
         <v>43</v>
       </c>
       <c r="C53" s="7"/>
@@ -2147,7 +2188,7 @@
       <c r="F53" s="7"/>
     </row>
     <row r="54" ht="23" customHeight="1" spans="1:6">
-      <c r="A54" s="27"/>
+      <c r="A54" s="26"/>
       <c r="B54" s="6" t="s">
         <v>44</v>
       </c>
@@ -2157,7 +2198,7 @@
       <c r="F54" s="7"/>
     </row>
     <row r="55" ht="23" customHeight="1" spans="1:6">
-      <c r="A55" s="27"/>
+      <c r="A55" s="26"/>
       <c r="B55" s="6" t="s">
         <v>45</v>
       </c>
@@ -2167,7 +2208,7 @@
       <c r="F55" s="7"/>
     </row>
     <row r="56" ht="23" customHeight="1" spans="1:6">
-      <c r="A56" s="27"/>
+      <c r="A56" s="26"/>
       <c r="B56" s="6" t="s">
         <v>46</v>
       </c>
@@ -2177,7 +2218,7 @@
       <c r="F56" s="7"/>
     </row>
     <row r="57" ht="23" customHeight="1" spans="1:6">
-      <c r="A57" s="27"/>
+      <c r="A57" s="26"/>
       <c r="B57" s="6" t="s">
         <v>47</v>
       </c>
@@ -2187,7 +2228,7 @@
       <c r="F57" s="7"/>
     </row>
     <row r="58" ht="23" customHeight="1" spans="1:6">
-      <c r="A58" s="27"/>
+      <c r="A58" s="26"/>
       <c r="B58" s="6" t="s">
         <v>48</v>
       </c>
@@ -2197,7 +2238,7 @@
       <c r="F58" s="7"/>
     </row>
     <row r="59" ht="23" customHeight="1" spans="1:6">
-      <c r="A59" s="27"/>
+      <c r="A59" s="26"/>
       <c r="B59" s="6" t="s">
         <v>49</v>
       </c>
@@ -2207,17 +2248,17 @@
       <c r="F59" s="7"/>
     </row>
     <row r="60" ht="23" customHeight="1" spans="1:6">
-      <c r="A60" s="27"/>
-      <c r="B60" s="32" t="s">
+      <c r="A60" s="26"/>
+      <c r="B60" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="C60" s="11"/>
+      <c r="C60" s="7"/>
       <c r="D60" s="7"/>
       <c r="E60" s="7"/>
       <c r="F60" s="7"/>
     </row>
     <row r="61" ht="23" customHeight="1" spans="1:6">
-      <c r="A61" s="28"/>
+      <c r="A61" s="27"/>
       <c r="B61" s="6"/>
       <c r="C61" s="7"/>
       <c r="D61" s="7"/>
@@ -2225,7 +2266,7 @@
       <c r="F61" s="7"/>
     </row>
     <row r="62" ht="23" customHeight="1" spans="1:6">
-      <c r="A62" s="26" t="s">
+      <c r="A62" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B62" s="6" t="s">
@@ -2237,7 +2278,7 @@
       <c r="F62" s="7"/>
     </row>
     <row r="63" ht="23" customHeight="1" spans="1:6">
-      <c r="A63" s="27"/>
+      <c r="A63" s="26"/>
       <c r="B63" s="6" t="s">
         <v>53</v>
       </c>
@@ -2247,7 +2288,7 @@
       <c r="F63" s="7"/>
     </row>
     <row r="64" ht="23" customHeight="1" spans="1:6">
-      <c r="A64" s="28"/>
+      <c r="A64" s="27"/>
       <c r="B64" s="7" t="s">
         <v>54</v>
       </c>
@@ -2257,34 +2298,34 @@
       <c r="F64" s="7"/>
     </row>
     <row r="65" ht="23" customHeight="1" spans="1:6">
-      <c r="A65" s="23" t="s">
+      <c r="A65" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="B65" s="23"/>
-      <c r="C65" s="23"/>
-      <c r="D65" s="23"/>
-      <c r="E65" s="30"/>
-      <c r="F65" s="30"/>
+      <c r="B65" s="22"/>
+      <c r="C65" s="22"/>
+      <c r="D65" s="22"/>
+      <c r="E65" s="28"/>
+      <c r="F65" s="28"/>
     </row>
     <row r="66" ht="23" customHeight="1" spans="1:6">
-      <c r="A66" s="23" t="s">
+      <c r="A66" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="B66" s="23"/>
-      <c r="C66" s="23"/>
-      <c r="D66" s="23"/>
-      <c r="E66" s="30"/>
-      <c r="F66" s="30"/>
+      <c r="B66" s="22"/>
+      <c r="C66" s="22"/>
+      <c r="D66" s="22"/>
+      <c r="E66" s="28"/>
+      <c r="F66" s="28"/>
     </row>
     <row r="67" ht="23" customHeight="1" spans="1:6">
-      <c r="A67" s="23" t="s">
+      <c r="A67" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="B67" s="23"/>
-      <c r="C67" s="23"/>
-      <c r="D67" s="23"/>
-      <c r="E67" s="30"/>
-      <c r="F67" s="30"/>
+      <c r="B67" s="22"/>
+      <c r="C67" s="22"/>
+      <c r="D67" s="22"/>
+      <c r="E67" s="28"/>
+      <c r="F67" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -2306,990 +2347,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:J67"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
-  <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="21.0666666666667" customWidth="1"/>
-    <col min="3" max="3" width="29.875" customWidth="1"/>
-    <col min="4" max="5" width="17.35" customWidth="1"/>
-    <col min="6" max="6" width="14.5" customWidth="1"/>
-    <col min="7" max="7" width="16.025" customWidth="1"/>
-    <col min="8" max="9" width="26.125" customWidth="1"/>
-    <col min="10" max="10" width="23.75" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="79" customHeight="1" spans="1:10">
-      <c r="A1" s="2"/>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-    </row>
-    <row r="2" s="1" customFormat="1" ht="29.25" spans="1:10">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" ht="26" customHeight="1" spans="1:10">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-    </row>
-    <row r="4" ht="26" customHeight="1" spans="1:10">
-      <c r="A4" s="5"/>
-      <c r="B4" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-    </row>
-    <row r="5" ht="26" customHeight="1" spans="1:10">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-    </row>
-    <row r="6" ht="26" customHeight="1" spans="1:10">
-      <c r="A6" s="5"/>
-      <c r="B6" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-    </row>
-    <row r="7" ht="26" customHeight="1" spans="1:10">
-      <c r="A7" s="5"/>
-      <c r="B7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-    </row>
-    <row r="8" ht="26" customHeight="1" spans="1:10">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-    </row>
-    <row r="9" ht="26" customHeight="1" spans="1:10">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-    </row>
-    <row r="10" ht="26" customHeight="1" spans="1:10">
-      <c r="A10" s="5"/>
-      <c r="B10" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-    </row>
-    <row r="11" ht="26" customHeight="1" spans="1:10">
-      <c r="A11" s="5"/>
-      <c r="B11" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-    </row>
-    <row r="12" ht="26" customHeight="1" spans="1:10">
-      <c r="A12" s="5"/>
-      <c r="B12" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-    </row>
-    <row r="13" ht="26" customHeight="1" spans="1:10">
-      <c r="A13" s="5"/>
-      <c r="B13" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-    </row>
-    <row r="14" ht="26" customHeight="1" spans="1:10">
-      <c r="A14" s="5"/>
-      <c r="B14" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-    </row>
-    <row r="15" ht="26" customHeight="1" spans="1:10">
-      <c r="A15" s="5"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-    </row>
-    <row r="16" ht="26" customHeight="1" spans="1:10">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-    </row>
-    <row r="17" ht="26" customHeight="1" spans="1:10">
-      <c r="A17" s="5"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-    </row>
-    <row r="18" ht="26" customHeight="1" spans="1:10">
-      <c r="A18" s="5"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-    </row>
-    <row r="19" ht="26" customHeight="1" spans="1:10">
-      <c r="A19" s="5"/>
-      <c r="B19" s="6"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-    </row>
-    <row r="20" ht="26" customHeight="1" spans="1:10">
-      <c r="A20" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-    </row>
-    <row r="21" ht="26" customHeight="1" spans="1:10">
-      <c r="A21" s="5"/>
-      <c r="B21" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
-    </row>
-    <row r="22" ht="26" customHeight="1" spans="1:10">
-      <c r="A22" s="5"/>
-      <c r="B22" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-    </row>
-    <row r="23" ht="26" customHeight="1" spans="1:10">
-      <c r="A23" s="5"/>
-      <c r="B23" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
-    </row>
-    <row r="24" ht="26" customHeight="1" spans="1:10">
-      <c r="A24" s="5"/>
-      <c r="B24" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-    </row>
-    <row r="25" ht="26" customHeight="1" spans="1:10">
-      <c r="A25" s="5"/>
-      <c r="B25" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
-    </row>
-    <row r="26" ht="26" customHeight="1" spans="1:10">
-      <c r="A26" s="5"/>
-      <c r="B26" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
-    </row>
-    <row r="27" ht="26" customHeight="1" spans="1:10">
-      <c r="A27" s="5"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-    </row>
-    <row r="28" ht="26" customHeight="1" spans="1:10">
-      <c r="A28" s="5"/>
-      <c r="B28" s="6"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="12"/>
-      <c r="I28" s="12"/>
-      <c r="J28" s="12"/>
-    </row>
-    <row r="29" ht="26" customHeight="1" spans="1:10">
-      <c r="A29" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
-      <c r="J29" s="8"/>
-    </row>
-    <row r="30" ht="26" customHeight="1" spans="1:10">
-      <c r="A30" s="14"/>
-      <c r="B30" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
-      <c r="G30" s="7"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="9"/>
-      <c r="J30" s="9"/>
-    </row>
-    <row r="31" ht="26" customHeight="1" spans="1:10">
-      <c r="A31" s="14"/>
-      <c r="B31" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="9"/>
-      <c r="J31" s="9"/>
-    </row>
-    <row r="32" ht="26" customHeight="1" spans="1:10">
-      <c r="A32" s="14"/>
-      <c r="B32" s="6"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="9"/>
-      <c r="I32" s="9"/>
-      <c r="J32" s="9"/>
-    </row>
-    <row r="33" ht="26" customHeight="1" spans="1:10">
-      <c r="A33" s="14"/>
-      <c r="B33" s="6"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="9"/>
-      <c r="I33" s="9"/>
-      <c r="J33" s="9"/>
-    </row>
-    <row r="34" ht="26" customHeight="1" spans="1:10">
-      <c r="A34" s="15"/>
-      <c r="B34" s="6"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
-      <c r="H34" s="12"/>
-      <c r="I34" s="12"/>
-      <c r="J34" s="12"/>
-    </row>
-    <row r="35" ht="26" customHeight="1" spans="1:10">
-      <c r="A35" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
-      <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="8"/>
-    </row>
-    <row r="36" ht="26" customHeight="1" spans="1:10">
-      <c r="A36" s="14"/>
-      <c r="B36" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="9"/>
-      <c r="J36" s="9"/>
-    </row>
-    <row r="37" ht="26" customHeight="1" spans="1:10">
-      <c r="A37" s="14"/>
-      <c r="B37" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="9"/>
-      <c r="I37" s="9"/>
-      <c r="J37" s="9"/>
-    </row>
-    <row r="38" ht="26" customHeight="1" spans="1:10">
-      <c r="A38" s="14"/>
-      <c r="B38" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
-      <c r="H38" s="9"/>
-      <c r="I38" s="9"/>
-      <c r="J38" s="9"/>
-    </row>
-    <row r="39" ht="26" customHeight="1" spans="1:10">
-      <c r="A39" s="14"/>
-      <c r="B39" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C39" s="7"/>
-      <c r="D39" s="7"/>
-      <c r="E39" s="7"/>
-      <c r="F39" s="7"/>
-      <c r="G39" s="7"/>
-      <c r="H39" s="9"/>
-      <c r="I39" s="9"/>
-      <c r="J39" s="9"/>
-    </row>
-    <row r="40" ht="26" customHeight="1" spans="1:10">
-      <c r="A40" s="14"/>
-      <c r="B40" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C40" s="7"/>
-      <c r="D40" s="7"/>
-      <c r="E40" s="7"/>
-      <c r="F40" s="7"/>
-      <c r="G40" s="7"/>
-      <c r="H40" s="9"/>
-      <c r="I40" s="9"/>
-      <c r="J40" s="9"/>
-    </row>
-    <row r="41" ht="26" customHeight="1" spans="1:10">
-      <c r="A41" s="14"/>
-      <c r="B41" s="6"/>
-      <c r="C41" s="7"/>
-      <c r="D41" s="7"/>
-      <c r="E41" s="7"/>
-      <c r="F41" s="7"/>
-      <c r="G41" s="7"/>
-      <c r="H41" s="9"/>
-      <c r="I41" s="9"/>
-      <c r="J41" s="9"/>
-    </row>
-    <row r="42" ht="26" customHeight="1" spans="1:10">
-      <c r="A42" s="14"/>
-      <c r="B42" s="6"/>
-      <c r="C42" s="7"/>
-      <c r="D42" s="7"/>
-      <c r="E42" s="7"/>
-      <c r="F42" s="7"/>
-      <c r="G42" s="7"/>
-      <c r="H42" s="9"/>
-      <c r="I42" s="9"/>
-      <c r="J42" s="9"/>
-    </row>
-    <row r="43" ht="26" customHeight="1" spans="1:10">
-      <c r="A43" s="14"/>
-      <c r="B43" s="6"/>
-      <c r="C43" s="7"/>
-      <c r="D43" s="7"/>
-      <c r="E43" s="7"/>
-      <c r="F43" s="7"/>
-      <c r="G43" s="7"/>
-      <c r="H43" s="9"/>
-      <c r="I43" s="9"/>
-      <c r="J43" s="9"/>
-    </row>
-    <row r="44" ht="26" customHeight="1" spans="1:10">
-      <c r="A44" s="14"/>
-      <c r="B44" s="6"/>
-      <c r="C44" s="7"/>
-      <c r="D44" s="7"/>
-      <c r="E44" s="7"/>
-      <c r="F44" s="7"/>
-      <c r="G44" s="7"/>
-      <c r="H44" s="9"/>
-      <c r="I44" s="9"/>
-      <c r="J44" s="9"/>
-    </row>
-    <row r="45" ht="26" customHeight="1" spans="1:10">
-      <c r="A45" s="14"/>
-      <c r="B45" s="6"/>
-      <c r="C45" s="7"/>
-      <c r="D45" s="7"/>
-      <c r="E45" s="7"/>
-      <c r="F45" s="7"/>
-      <c r="G45" s="7"/>
-      <c r="H45" s="9"/>
-      <c r="I45" s="9"/>
-      <c r="J45" s="9"/>
-    </row>
-    <row r="46" ht="26" customHeight="1" spans="1:10">
-      <c r="A46" s="14"/>
-      <c r="B46" s="6"/>
-      <c r="C46" s="7"/>
-      <c r="D46" s="7"/>
-      <c r="E46" s="7"/>
-      <c r="F46" s="7"/>
-      <c r="G46" s="7"/>
-      <c r="H46" s="9"/>
-      <c r="I46" s="9"/>
-      <c r="J46" s="9"/>
-    </row>
-    <row r="47" ht="26" customHeight="1" spans="1:10">
-      <c r="A47" s="15"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="7"/>
-      <c r="F47" s="7"/>
-      <c r="G47" s="7"/>
-      <c r="H47" s="12"/>
-      <c r="I47" s="12"/>
-      <c r="J47" s="12"/>
-    </row>
-    <row r="48" ht="26" customHeight="1" spans="1:10">
-      <c r="A48" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C48" s="7"/>
-      <c r="D48" s="7"/>
-      <c r="E48" s="7"/>
-      <c r="F48" s="7"/>
-      <c r="G48" s="7"/>
-      <c r="H48" s="8"/>
-      <c r="I48" s="8"/>
-      <c r="J48" s="8"/>
-    </row>
-    <row r="49" ht="26" customHeight="1" spans="1:10">
-      <c r="A49" s="14"/>
-      <c r="B49" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C49" s="7"/>
-      <c r="D49" s="7"/>
-      <c r="E49" s="7"/>
-      <c r="F49" s="7"/>
-      <c r="G49" s="7"/>
-      <c r="H49" s="9"/>
-      <c r="I49" s="9"/>
-      <c r="J49" s="9"/>
-    </row>
-    <row r="50" ht="26" customHeight="1" spans="1:10">
-      <c r="A50" s="14"/>
-      <c r="B50" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="7"/>
-      <c r="F50" s="7"/>
-      <c r="G50" s="7"/>
-      <c r="H50" s="9"/>
-      <c r="I50" s="9"/>
-      <c r="J50" s="9"/>
-    </row>
-    <row r="51" ht="26" customHeight="1" spans="1:10">
-      <c r="A51" s="14"/>
-      <c r="B51" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C51" s="7"/>
-      <c r="D51" s="7"/>
-      <c r="E51" s="7"/>
-      <c r="F51" s="7"/>
-      <c r="G51" s="7"/>
-      <c r="H51" s="9"/>
-      <c r="I51" s="9"/>
-      <c r="J51" s="9"/>
-    </row>
-    <row r="52" ht="26" customHeight="1" spans="1:10">
-      <c r="A52" s="15"/>
-      <c r="B52" s="6"/>
-      <c r="C52" s="7"/>
-      <c r="D52" s="7"/>
-      <c r="E52" s="7"/>
-      <c r="F52" s="7"/>
-      <c r="G52" s="7"/>
-      <c r="H52" s="12"/>
-      <c r="I52" s="12"/>
-      <c r="J52" s="12"/>
-    </row>
-    <row r="53" ht="26" customHeight="1" spans="1:10">
-      <c r="A53" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="B53" s="31" t="s">
-        <v>43</v>
-      </c>
-      <c r="C53" s="7"/>
-      <c r="D53" s="7"/>
-      <c r="E53" s="7"/>
-      <c r="F53" s="7"/>
-      <c r="G53" s="7"/>
-      <c r="H53" s="8"/>
-      <c r="I53" s="8"/>
-      <c r="J53" s="8"/>
-    </row>
-    <row r="54" ht="26" customHeight="1" spans="1:10">
-      <c r="A54" s="14"/>
-      <c r="B54" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C54" s="7"/>
-      <c r="D54" s="7"/>
-      <c r="E54" s="7"/>
-      <c r="F54" s="7"/>
-      <c r="G54" s="7"/>
-      <c r="H54" s="9"/>
-      <c r="I54" s="9"/>
-      <c r="J54" s="9"/>
-    </row>
-    <row r="55" ht="26" customHeight="1" spans="1:10">
-      <c r="A55" s="14"/>
-      <c r="B55" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C55" s="7"/>
-      <c r="D55" s="7"/>
-      <c r="E55" s="7"/>
-      <c r="F55" s="7"/>
-      <c r="G55" s="7"/>
-      <c r="H55" s="9"/>
-      <c r="I55" s="9"/>
-      <c r="J55" s="9"/>
-    </row>
-    <row r="56" ht="26" customHeight="1" spans="1:10">
-      <c r="A56" s="14"/>
-      <c r="B56" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C56" s="7"/>
-      <c r="D56" s="7"/>
-      <c r="E56" s="7"/>
-      <c r="F56" s="7"/>
-      <c r="G56" s="7"/>
-      <c r="H56" s="9"/>
-      <c r="I56" s="9"/>
-      <c r="J56" s="9"/>
-    </row>
-    <row r="57" ht="26" customHeight="1" spans="1:10">
-      <c r="A57" s="14"/>
-      <c r="B57" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C57" s="7"/>
-      <c r="D57" s="7"/>
-      <c r="E57" s="7"/>
-      <c r="F57" s="7"/>
-      <c r="G57" s="7"/>
-      <c r="H57" s="9"/>
-      <c r="I57" s="9"/>
-      <c r="J57" s="9"/>
-    </row>
-    <row r="58" ht="26" customHeight="1" spans="1:10">
-      <c r="A58" s="14"/>
-      <c r="B58" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C58" s="7"/>
-      <c r="D58" s="7"/>
-      <c r="E58" s="7"/>
-      <c r="F58" s="7"/>
-      <c r="G58" s="7"/>
-      <c r="H58" s="9"/>
-      <c r="I58" s="9"/>
-      <c r="J58" s="9"/>
-    </row>
-    <row r="59" ht="26" customHeight="1" spans="1:10">
-      <c r="A59" s="14"/>
-      <c r="B59" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C59" s="7"/>
-      <c r="D59" s="7"/>
-      <c r="E59" s="7"/>
-      <c r="F59" s="7"/>
-      <c r="G59" s="7"/>
-      <c r="H59" s="9"/>
-      <c r="I59" s="9"/>
-      <c r="J59" s="9"/>
-    </row>
-    <row r="60" ht="26" customHeight="1" spans="1:10">
-      <c r="A60" s="14"/>
-      <c r="B60" s="33" t="s">
-        <v>50</v>
-      </c>
-      <c r="C60" s="11"/>
-      <c r="D60" s="7"/>
-      <c r="E60" s="7"/>
-      <c r="F60" s="7"/>
-      <c r="G60" s="7"/>
-      <c r="H60" s="9"/>
-      <c r="I60" s="9"/>
-      <c r="J60" s="9"/>
-    </row>
-    <row r="61" ht="26" customHeight="1" spans="1:10">
-      <c r="A61" s="15"/>
-      <c r="B61" s="6"/>
-      <c r="C61" s="7"/>
-      <c r="D61" s="7"/>
-      <c r="E61" s="7"/>
-      <c r="F61" s="7"/>
-      <c r="G61" s="7"/>
-      <c r="H61" s="12"/>
-      <c r="I61" s="12"/>
-      <c r="J61" s="12"/>
-    </row>
-    <row r="62" ht="26" customHeight="1" spans="1:10">
-      <c r="A62" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C62" s="7"/>
-      <c r="D62" s="7"/>
-      <c r="E62" s="7"/>
-      <c r="F62" s="7"/>
-      <c r="G62" s="7"/>
-      <c r="H62" s="8"/>
-      <c r="I62" s="8"/>
-      <c r="J62" s="8"/>
-    </row>
-    <row r="63" ht="26" customHeight="1" spans="1:10">
-      <c r="A63" s="14"/>
-      <c r="B63" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C63" s="7"/>
-      <c r="D63" s="7"/>
-      <c r="E63" s="7"/>
-      <c r="F63" s="7"/>
-      <c r="G63" s="7"/>
-      <c r="H63" s="9"/>
-      <c r="I63" s="9"/>
-      <c r="J63" s="9"/>
-    </row>
-    <row r="64" ht="26" customHeight="1" spans="1:10">
-      <c r="A64" s="15"/>
-      <c r="B64" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C64" s="7"/>
-      <c r="D64" s="7"/>
-      <c r="E64" s="7"/>
-      <c r="F64" s="7"/>
-      <c r="G64" s="7"/>
-      <c r="H64" s="12"/>
-      <c r="I64" s="12"/>
-      <c r="J64" s="12"/>
-    </row>
-    <row r="65" ht="48" customHeight="1" spans="1:10">
-      <c r="A65" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B65" s="17"/>
-      <c r="C65" s="17"/>
-      <c r="D65" s="17"/>
-      <c r="E65" s="17"/>
-      <c r="F65" s="17"/>
-      <c r="G65" s="18"/>
-      <c r="H65" s="19"/>
-      <c r="I65" s="20"/>
-      <c r="J65" s="20"/>
-    </row>
-    <row r="66" ht="48" customHeight="1" spans="1:10">
-      <c r="A66" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B66" s="17"/>
-      <c r="C66" s="17"/>
-      <c r="D66" s="17"/>
-      <c r="E66" s="17"/>
-      <c r="F66" s="17"/>
-      <c r="G66" s="18"/>
-      <c r="H66" s="19"/>
-      <c r="I66" s="20"/>
-      <c r="J66" s="20"/>
-    </row>
-    <row r="67" ht="48" customHeight="1" spans="1:10">
-      <c r="A67" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="B67" s="21"/>
-      <c r="C67" s="21"/>
-      <c r="D67" s="21"/>
-      <c r="E67" s="21"/>
-      <c r="F67" s="21"/>
-      <c r="G67" s="21"/>
-      <c r="H67" s="19"/>
-      <c r="I67" s="20"/>
-      <c r="J67" s="20"/>
-    </row>
-  </sheetData>
-  <mergeCells count="32">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A65:G65"/>
-    <mergeCell ref="A66:G66"/>
-    <mergeCell ref="A67:G67"/>
-    <mergeCell ref="A3:A19"/>
-    <mergeCell ref="A20:A28"/>
-    <mergeCell ref="A29:A34"/>
-    <mergeCell ref="A35:A47"/>
-    <mergeCell ref="A48:A52"/>
-    <mergeCell ref="A53:A61"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="H3:H19"/>
-    <mergeCell ref="H20:H28"/>
-    <mergeCell ref="H29:H34"/>
-    <mergeCell ref="H35:H47"/>
-    <mergeCell ref="H48:H52"/>
-    <mergeCell ref="H53:H61"/>
-    <mergeCell ref="H62:H64"/>
-    <mergeCell ref="I3:I19"/>
-    <mergeCell ref="I20:I28"/>
-    <mergeCell ref="I29:I34"/>
-    <mergeCell ref="I35:I47"/>
-    <mergeCell ref="I48:I52"/>
-    <mergeCell ref="I53:I61"/>
-    <mergeCell ref="I62:I64"/>
-    <mergeCell ref="J3:J19"/>
-    <mergeCell ref="J20:J28"/>
-    <mergeCell ref="J29:J34"/>
-    <mergeCell ref="J35:J47"/>
-    <mergeCell ref="J48:J52"/>
-    <mergeCell ref="J53:J61"/>
-    <mergeCell ref="J62:J64"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
 </file>
</xml_diff>